<commit_message>
Complete Milestone 3 features
</commit_message>
<xml_diff>
--- a/Agile/Defect_Tracker Template_v0.1.xlsx
+++ b/Agile/Defect_Tracker Template_v0.1.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GeethaJyothi\.gemini\antigravity\scratch\knowledge-retrieval-platform\Agile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1529751A-99C4-4233-8104-CEB3E356847C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4830"/>
   </bookViews>
   <sheets>
     <sheet name="Defects" sheetId="1" r:id="rId1"/>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
   <si>
     <t>Sl No</t>
   </si>
@@ -69,13 +68,49 @@
   </si>
   <si>
     <t>Status(Open/Closed)</t>
+  </si>
+  <si>
+    <t>Geetha</t>
+  </si>
+  <si>
+    <t>Milestone 2 multi-agent functionality required integration with the existing Milestone 1 RAG flow.</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Integrated the new agents through the Multi-Agent Orchestrator and standardized the flow.</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Resolved during M2 integration.</t>
+  </si>
+  <si>
+    <t>Ambiguous queries needed to be prevented from entering normal retrieval without sufficient context.</t>
+  </si>
+  <si>
+    <t>Added ambiguous-query classification and routing so normal retrieval is skipped for the M2 ambiguous path.</t>
+  </si>
+  <si>
+    <t>Interactive clarification remains Milestone 3.</t>
+  </si>
+  <si>
+    <t>Retrieved content could be insufficiently relevant for an out-of-domain query.</t>
+  </si>
+  <si>
+    <t>Added relevance/groundedness validation so unsupported retrieval is not treated as valid evidence.</t>
+  </si>
+  <si>
+    <t>Supports grounded response behavior.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -132,6 +167,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF003366"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -147,7 +188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -170,11 +211,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -191,6 +247,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -284,23 +343,6 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -336,23 +378,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -528,7 +553,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -544,7 +569,7 @@
     <col min="12" max="16384" width="17.5703125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="32.25" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,44 +604,98 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+    <row r="2" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
@@ -834,11 +913,11 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1:G1048576</xm:sqref>
+          <xm:sqref>G1 G5:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -847,7 +926,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -883,6 +962,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1014,22 +1108,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1045,21 +1141,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Milestone 4 Complete: Query Analytics, Knowledge Gap Detection, Multi-Domain Evaluation, Smart Answer Synthesis, and UI Transparency Enhancements
</commit_message>
<xml_diff>
--- a/Agile/Defect_Tracker Template_v0.1.xlsx
+++ b/Agile/Defect_Tracker Template_v0.1.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4830"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4830"/>
   </bookViews>
   <sheets>
     <sheet name="Defects" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="40">
   <si>
     <t>Sl No</t>
   </si>
@@ -73,44 +73,83 @@
     <t>Geetha</t>
   </si>
   <si>
-    <t>Milestone 2 multi-agent functionality required integration with the existing Milestone 1 RAG flow.</t>
-  </si>
-  <si>
     <t>Sprint 2</t>
   </si>
   <si>
-    <t>Integrated the new agents through the Multi-Agent Orchestrator and standardized the flow.</t>
-  </si>
-  <si>
     <t>Closed</t>
   </si>
   <si>
-    <t>Resolved during M2 integration.</t>
-  </si>
-  <si>
-    <t>Ambiguous queries needed to be prevented from entering normal retrieval without sufficient context.</t>
-  </si>
-  <si>
-    <t>Added ambiguous-query classification and routing so normal retrieval is skipped for the M2 ambiguous path.</t>
-  </si>
-  <si>
-    <t>Interactive clarification remains Milestone 3.</t>
-  </si>
-  <si>
-    <t>Retrieved content could be insufficiently relevant for an out-of-domain query.</t>
-  </si>
-  <si>
-    <t>Added relevance/groundedness validation so unsupported retrieval is not treated as valid evidence.</t>
-  </si>
-  <si>
-    <t>Supports grounded response behavior.</t>
+    <t>Document parsing failed to handle different text extraction behavior consistently across supported file types.</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>Added file-type-specific extraction and normalized the extracted text.</t>
+  </si>
+  <si>
+    <t>Verified with supported PDF, DOCX, TXT and CSV samples.</t>
+  </si>
+  <si>
+    <t>Ambiguous queries were entering the normal retrieval path without enough context.</t>
+  </si>
+  <si>
+    <t>Added query classification and routing for ambiguous requests.</t>
+  </si>
+  <si>
+    <t>Handled through the Query Understanding Agent.</t>
+  </si>
+  <si>
+    <t>Low-relevance retrieved chunks could still be passed to response generation.</t>
+  </si>
+  <si>
+    <t>Added relevance filtering before grounded response generation.</t>
+  </si>
+  <si>
+    <t>Unsupported evidence is no longer treated as valid context.</t>
+  </si>
+  <si>
+    <t>Follow-up questions did not consistently retain the previous turn's context.</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Added conversation-memory handling to preserve recent turns.</t>
+  </si>
+  <si>
+    <t>Validated with multi-turn question sequences.</t>
+  </si>
+  <si>
+    <t>Voice input depended on browser permission and recognition availability.</t>
+  </si>
+  <si>
+    <t>Added permission handling and a text-input fallback.</t>
+  </si>
+  <si>
+    <t>Fallback is available when speech recognition is unavailable.</t>
+  </si>
+  <si>
+    <t>Analytics records did not initially capture enough information to identify knowledge gaps.</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>Standardized query type, confidence, retrieval and resolution fields.</t>
+  </si>
+  <si>
+    <t>Supports unanswered and low-confidence analysis.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="dd\-mm\-yyyy"/>
+  </numFmts>
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -173,6 +212,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -188,7 +233,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -226,11 +271,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -247,8 +307,23 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,19 +679,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="64.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="8"/>
+      <c r="C2" s="9">
+        <v>46257</v>
+      </c>
       <c r="D2" s="8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>16</v>
@@ -625,29 +702,33 @@
         <v>9</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="8"/>
+        <v>21</v>
+      </c>
+      <c r="I2" s="9">
+        <v>46258</v>
+      </c>
       <c r="J2" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="64.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="9">
+        <v>46263</v>
+      </c>
       <c r="D3" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>16</v>
@@ -656,29 +737,33 @@
         <v>9</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="8"/>
+        <v>24</v>
+      </c>
+      <c r="I3" s="9">
+        <v>46264</v>
+      </c>
       <c r="J3" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="95.25" thickBot="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="64.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="8"/>
+      <c r="C4" s="9">
+        <v>46266</v>
+      </c>
       <c r="D4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>16</v>
@@ -687,54 +772,122 @@
         <v>9</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="8"/>
+        <v>27</v>
+      </c>
+      <c r="I4" s="9">
+        <v>46267</v>
+      </c>
       <c r="J4" s="8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="6"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="64.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="11">
+        <v>46270</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="11">
+        <v>46272</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="79.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="11">
+        <v>46274</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="11">
+        <v>46275</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="63.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="13">
+        <v>46287</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="11">
+        <v>46289</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
@@ -917,7 +1070,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1 G5:G1048576</xm:sqref>
+          <xm:sqref>G1 G8:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -962,21 +1115,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1108,24 +1246,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1141,4 +1277,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>